<commit_message>
Track PHS6 housing M6 capture in Rev F review BOM
</commit_message>
<xml_diff>
--- a/outputs/20261002_reve_upper_pocket_bom/2026_BIZ-Lab_재료비관리_RevF_상부포켓검토.xlsx
+++ b/outputs/20261002_reve_upper_pocket_bom/2026_BIZ-Lab_재료비관리_RevF_상부포켓검토.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R89f0d587c2c74c9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R2e682456d53845ac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3380,7 +3380,7 @@
       </x:c>
       <x:c r="I73" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">UP01A/B/C 및 신규 핀·리테이너·볼트/T너트·스페이서 미견적. 최종 예산 판정 UNKNOWN; 발주 보류.</x:t>
+          <x:t xml:space="preserve">UP01A/B/C 및 신규 핀·핀 리테이너·PHS6 하우징 M6 이탈방지품·장착 볼트/T너트·스페이서 미견적. 최종 예산 판정 UNKNOWN; 발주 보류.</x:t>
         </x:is>
       </x:c>
       <x:c r="M73" s="1" t="n"/>
@@ -3630,7 +3630,47 @@
       </x:c>
       <x:c r="M80" s="1" t="n"/>
     </x:row>
-    <x:row r="81" s="13" customFormat="1" ht="16.5" customHeight="1">
+    <x:row r="81" s="13" customFormat="1" ht="38" customHeight="1">
+      <x:c r="B81" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PHS6 하우징 M6 포획·이탈방지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C81" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">하우징 M6 유효물림·잠금 방식</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D81" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미선정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E81" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">3축 총수량/포장 미확정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F81" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미확정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G81" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">—</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H81" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">견적 미확정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I81" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">정확 SKU·3축 수량·M6 유효물림·잠금 방식·납기·카드결제 확인 전 HOLD</x:t>
+        </x:is>
+      </x:c>
       <x:c r="M81" s="1" t="n"/>
     </x:row>
     <x:row r="82" s="13" customFormat="1" ht="16.5" customHeight="1">
@@ -10023,69 +10063,69 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="R77019f8e8d514cc1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="R6cd3db247e064d5c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R3e899b83b8ea47ee"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="R89526c1409e0468c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="Re45c0cdcb7244ef7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="R78dfa373ddaf4cdf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="R6ad9a121c8d040cf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="Ra2a8cb537a7c4253"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="R7255b6ccf92d4428"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="R48b19a6599e44a38"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="R9d4ad45df50e44d8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="Ra01cfc9f2f634c35"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="Rd2d394ce8be54192"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="R565cc2f9ca734226"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="R32b7c9e01d8d4eca"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="Rcf5665432f7648e9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="Ra6606855d9954821"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="Rd56816c8576c428e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="R5c604eb0c2c34997"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="Rb8dfb6c4012b4448"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="R2a1dc2c90071457e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="R9ad11fa440974445"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="R7cd00d6e9baa49c5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="R23c456ed05f04f89"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="R8fc038d1b54e4fe3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="R9f2f87a04e934b23"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="Rc395ac39d46f48d0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="Ref9c487e4549495a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="R4e05e2a6dc2a40d4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="R0b4b9525d5ea4258"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="Re19b7adcfb3147d6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="R33bbd29c56bf4b41"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="Rdba3af23fc8942bb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="R755d34bd63ba4142"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="Rf5c984e96a3641ed"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="Ra42b80d60b90411e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="R8c69b8b789d04ffc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="R7c2d6ea5dbac43d8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="R0dfd529f6e2c41ca"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="R1157308004334823"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="R1ba2a46bf6954fa2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="Ra73976c75f9a46e1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="Rc20aba1e210944c7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="R12523928fbe84200"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="R6fa64ccd3c694a10"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="R64112fda2b2a40cd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="R566c52ae2f674f0c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="R24cad71a092749e8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="Rb53fdb1f0a0b4fd5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="R2afbfca104cc4ef1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="Rb03370f9d8764b1b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="Rf5731f4d8b89486a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="R4a6bf617877944ae"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="Rdff5794ae8554938"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="R029d187a60754285"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="Rce10375b3c564866"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="R9a135708fef64a02"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="R4b88d54e51854085"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="R7ad99e72c83c4e5d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="Raa908458deff4335"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="Rba3116cc733e460e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="R14a30a67d3d44847"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="R04e207b0804d4900"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="R0d97cafe548a4fe6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="R3ee3c0a924c0472e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R26207aa69f224e4b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="R2a1d3a7b63784492"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="R36e7c1b021004998"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="R6b4429bab7fe45a3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="Re2ac3fa9eaa2478b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="R40af45065fa14ac4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="R49baa0434b8e4369"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="Raa97b81db1e8460f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="R9b20cf4220374446"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="R0dbcb27f8d6b4771"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="R3e01bc86a01f4bee"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="Re42b7d6f07ff4d3b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="R4c61de3661bf4c2c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="Rc18fa2a2fd834959"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="Rf0c0c35dc0cf429d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="Rdf7bbf20033f41ab"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="Rb4fbcc9afe014b1b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="Rb057239801ff4963"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="Rc561cda471c34224"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="R6b4094d8b36f4ec8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="Re2f463ac2bbb4766"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="Rf9f54879e0ed489f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="R85104603bce448d1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="Rc971ca4403074def"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="R0f019311b3e54861"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="R541351a1b09d4a0c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="Rf84a33b6a34b4dce"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="R52f2e4357a9b4ea4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R80046d3654684952"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="Rff449dae20a74231"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="R34899b65de0848e9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="Rfaf7575f3f1243f6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="R3257ebc43ee841c6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="Rdee3c2d1c20d4c51"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="Rc3d1d2c8526d48a1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="Redb5e7dd00b74067"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="R3094240250e546c6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="R142149ceca404b57"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="R0bd7996d44b34bcf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="Rfeb97616eef24230"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="Rba1a2f36eb154e3b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="R829eafceca0a47a1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="Re53b359504b44574"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="R589ed1d67f064ff7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="Rd8dec4f606f54fc2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="R7181e09967f9457e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="Re74b8c8d1c374897"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="R5d33b7d71b904bab"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="R89cf9888477f4c48"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="R97b1362f86464574"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="R1ff8ebdaa82c4386"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="Rf8524587a35a4995"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="Rf6ff64e335b54228"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="R8413f2d245864b9f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="R7e49e34720604698"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="R509d0b6145b64750"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="R540f57d9873b4296"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="R495bc5c4a7754759"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="R35ca62b371704712"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="Rb7ca1dadffd441a9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="R1e726436591949da"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Clarify Rev F upper joint BOM hold candidates
</commit_message>
<xml_diff>
--- a/outputs/20261002_reve_upper_pocket_bom/2026_BIZ-Lab_재료비관리_RevF_상부포켓검토.xlsx
+++ b/outputs/20261002_reve_upper_pocket_bom/2026_BIZ-Lab_재료비관리_RevF_상부포켓검토.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R2e682456d53845ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R1945be0e69a148e9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -195,7 +195,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="38">
+  <x:cellXfs count="39">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -306,6 +306,9 @@
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2898,7 +2901,7 @@
           <x:t xml:space="preserve">견적 미확정</x:t>
         </x:is>
       </x:c>
-      <x:c r="I59" s="24" t="inlineStr">
+      <x:c r="I59" s="38" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">UP01A. 축 A 단품 1개. S45C/SM45C 가공 완료품 견적 후보; STEP/도면 승인, 업체 수락, 공급가·VAT·납기·결제 확인 전 발주 보류.</x:t>
         </x:is>
@@ -2936,7 +2939,7 @@
           <x:t xml:space="preserve">견적 미확정</x:t>
         </x:is>
       </x:c>
-      <x:c r="I60" s="24" t="inlineStr">
+      <x:c r="I60" s="38" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">UP01B. 축 B 단품 1개. S45C/SM45C 가공 완료품 견적 후보; STEP/도면 승인, 업체 수락, 공급가·VAT·납기·결제 확인 전 발주 보류.</x:t>
         </x:is>
@@ -2974,7 +2977,7 @@
           <x:t xml:space="preserve">견적 미확정</x:t>
         </x:is>
       </x:c>
-      <x:c r="I61" s="24" t="inlineStr">
+      <x:c r="I61" s="38" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">UP01C. 축 C 단품 1개. S45C/SM45C 가공 완료품 견적 후보; STEP/도면 승인, 업체 수락, 공급가·VAT·납기·결제 확인 전 발주 보류.</x:t>
         </x:is>
@@ -3362,7 +3365,7 @@
       </x:c>
       <x:c r="M72" s="1" t="n"/>
     </x:row>
-    <x:row r="73" s="13" customFormat="1" ht="16.5" customHeight="1">
+    <x:row r="73" s="13" customFormat="1" ht="54" customHeight="1">
       <x:c r="A73" t="n"/>
       <x:c r="B73" t="inlineStr">
         <x:is>
@@ -3378,9 +3381,9 @@
         <x:f>$I$2-H72</x:f>
         <x:v>867964</x:v>
       </x:c>
-      <x:c r="I73" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">UP01A/B/C 및 신규 핀·핀 리테이너·PHS6 하우징 M6 이탈방지품·장착 볼트/T너트·스페이서 미견적. 최종 예산 판정 UNKNOWN; 발주 보류.</x:t>
+      <x:c r="I73" s="38" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">UP01A/B/C 및 신규 핀·와셔·PHS6 M6·장착 볼트/T너트 미견적. E링은 HCDGH 동봉(별도 구매 없음). 최종 예산 적합 UNKNOWN; 구매 보류.</x:t>
         </x:is>
       </x:c>
       <x:c r="M73" s="1" t="n"/>
@@ -3410,7 +3413,7 @@
       <x:c r="H75" s="31" t="n"/>
       <x:c r="I75" s="31" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">미등재·HOLD</x:t>
+          <x:t xml:space="preserve">유료 구매행 미반영·HOLD</x:t>
         </x:is>
       </x:c>
       <x:c r="M75" s="1" t="n"/>
@@ -3458,7 +3461,7 @@
       </x:c>
       <x:c r="M76" s="1" t="n"/>
     </x:row>
-    <x:row r="77" s="13" customFormat="1" ht="38" customHeight="1">
+    <x:row r="77" s="13" customFormat="1" ht="52" customHeight="1">
       <x:c r="B77" s="33" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">신규 상부 피벗 핀</x:t>
@@ -3471,204 +3474,204 @@
       </x:c>
       <x:c r="D77" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">미선정</x:t>
+          <x:t xml:space="preserve">미선정 (후보 HCDGH6-35)</x:t>
         </x:is>
       </x:c>
       <x:c r="E77" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">길이/수량 미확정</x:t>
+          <x:t xml:space="preserve">3개(축당 1개), E링 각 1개 동봉</x:t>
         </x:is>
       </x:c>
       <x:c r="F77" s="33" t="inlineStr">
         <x:is>
+          <x:t xml:space="preserve">한국미스미</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G77" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://kr.misumi-ec.com/vona2/detail/110300095750/?HissuCode=HCDGH6-35</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H77" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">견적 미확정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I77" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">핀 보증 항복·홈 강도·eye 공차·링 축하중 미검증 HOLD</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M77" s="1" t="n"/>
+    </x:row>
+    <x:row r="78" s="13" customFormat="1" ht="52" customHeight="1">
+      <x:c r="B78" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">핀 리테이너</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C78" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">피벗 축방향 이탈 방지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D78" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">HCDGH6-35 동봉 E형 No.5 고정링</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E78" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">동봉 3개; 별도 발주 없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F78" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">한국미스미</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G78" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://kr.misumi-ec.com/vona2/detail/110300095750/?HissuCode=HCDGH6-35</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H78" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">동봉 (별도 발주 없음)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I78" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">HCDGH에 동봉; 별도 구매 0. 실제 링 유지력 미검증 HOLD</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M78" s="1" t="n"/>
+    </x:row>
+    <x:row r="79" s="13" customFormat="1" ht="52" customHeight="1">
+      <x:c r="B79" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">조립 스페이서/와셔</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C79" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">축별 유격·간섭 제어</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D79" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미선정 (후보 WSSB10-6-4; F09 CIMR6-12-0.5)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E79" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">와셔 3개; 심 명목 9장(기존 F09 12장 후보)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F79" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">한국미스미</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G79" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://kr.misumi-ec.com/vona2/detail/110302677010/?HissuCode=WSSB10-6-4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H79" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">신규 와셔 견적 미확정; F09 기포함</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I79" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">eye 폭·링 장착 여유 미확정. F09 심 12장과 중복 구매 금지 HOLD</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M79" s="1" t="n"/>
+    </x:row>
+    <x:row r="80" s="13" customFormat="1" ht="52" customHeight="1">
+      <x:c r="B80" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PHS6 하우징 M6 포획·이탈방지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C80" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">하우징 M6 유효물림·잠금 방식</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D80" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미선정 (후보 PACK-SCB6-12-YBM)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E80" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">3축 3개 필요; 후보 10개입 1팩</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F80" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">한국미스미</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G80" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://kr.misumi-ec.com/vona2/detail/110300239250/?HissuCode=PACK-SCB6-12-YBM</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H80" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">견적 미확정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I80" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F21/G9EA용 볼트와 구별. M6 유효물림·잠금·머리 여유·카드결제 HOLD</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M80" s="1" t="n"/>
+    </x:row>
+    <x:row r="81" s="13" customFormat="1" ht="52" customHeight="1">
+      <x:c r="B81" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">브래킷 장착 볼트·T너트</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C81" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">3030 프레임에 3개 브래킷 장착</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D81" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미선정 (F02/F07 재사용 미확정)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E81" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">명목 볼트 6개·너트 6개; 길이·포장 미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F81" s="33" t="inlineStr">
+        <x:is>
           <x:t xml:space="preserve">미확정</x:t>
         </x:is>
       </x:c>
-      <x:c r="G77" s="33" t="inlineStr">
+      <x:c r="G81" s="33" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">—</x:t>
         </x:is>
       </x:c>
-      <x:c r="H77" s="33" t="inlineStr">
+      <x:c r="H81" s="33" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">견적 미확정</x:t>
         </x:is>
       </x:c>
-      <x:c r="I77" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Task6 형상/공차 및 유지 방식 확인 전 HOLD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M77" s="1" t="n"/>
-    </x:row>
-    <x:row r="78" s="13" customFormat="1" ht="38" customHeight="1">
-      <x:c r="B78" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">핀 리테이너</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C78" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">피벗 축방향 이탈 방지</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D78" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">미선정</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E78" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">미확정</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F78" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">미확정</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G78" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">—</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H78" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">견적 미확정</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I78" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">캡/와셔/나사 방식 확정 전 HOLD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M78" s="1" t="n"/>
-    </x:row>
-    <x:row r="79" s="13" customFormat="1" ht="38" customHeight="1">
-      <x:c r="B79" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">브래킷 장착 볼트·T너트</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C79" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">3030 프레임에 3개 브래킷 장착</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D79" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">미선정</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E79" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">길이·체결점/포장 미확정</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F79" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">미확정</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G79" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">—</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H79" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">견적 미확정</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I79" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">실제 프로파일 슬롯·브래킷 두께/체결점 검증 전 HOLD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M79" s="1" t="n"/>
-    </x:row>
-    <x:row r="80" s="13" customFormat="1" ht="38" customHeight="1">
-      <x:c r="B80" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">조립 스페이서/와셔</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C80" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">축별 유격·간섭 제어</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D80" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">미선정</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E80" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">두께/수량 미확정</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F80" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">미확정</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G80" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">—</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H80" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">견적 미확정</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I80" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">F09 기존 용도와 별도 판정 전 HOLD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M80" s="1" t="n"/>
-    </x:row>
-    <x:row r="81" s="13" customFormat="1" ht="38" customHeight="1">
-      <x:c r="B81" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">PHS6 하우징 M6 포획·이탈방지</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C81" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">하우징 M6 유효물림·잠금 방식</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D81" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">미선정</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E81" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">3축 총수량/포장 미확정</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F81" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">미확정</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G81" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">—</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H81" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">견적 미확정</x:t>
-        </x:is>
-      </x:c>
       <x:c r="I81" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">정확 SKU·3축 수량·M6 유효물림·잠금 방식·납기·카드결제 확인 전 HOLD</x:t>
+          <x:t xml:space="preserve">F02/F07 자동 전용 금지. 납품 3030 슬롯·체결력 검증 전 HOLD</x:t>
         </x:is>
       </x:c>
       <x:c r="M81" s="1" t="n"/>
@@ -10063,69 +10066,73 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="R0d97cafe548a4fe6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="R3ee3c0a924c0472e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R26207aa69f224e4b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="R2a1d3a7b63784492"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="R36e7c1b021004998"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="R6b4429bab7fe45a3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="Re2ac3fa9eaa2478b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="R40af45065fa14ac4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="R49baa0434b8e4369"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="Raa97b81db1e8460f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="R9b20cf4220374446"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="R0dbcb27f8d6b4771"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="R3e01bc86a01f4bee"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="Re42b7d6f07ff4d3b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="R4c61de3661bf4c2c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="Rc18fa2a2fd834959"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="Rf0c0c35dc0cf429d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="Rdf7bbf20033f41ab"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="Rb4fbcc9afe014b1b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="Rb057239801ff4963"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="Rc561cda471c34224"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="R6b4094d8b36f4ec8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="Re2f463ac2bbb4766"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="Rf9f54879e0ed489f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="R85104603bce448d1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="Rc971ca4403074def"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="R0f019311b3e54861"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="R541351a1b09d4a0c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="Rf84a33b6a34b4dce"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="R52f2e4357a9b4ea4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R80046d3654684952"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="Rff449dae20a74231"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="R34899b65de0848e9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="Rfaf7575f3f1243f6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="R3257ebc43ee841c6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="Rdee3c2d1c20d4c51"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="Rc3d1d2c8526d48a1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="Redb5e7dd00b74067"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="R3094240250e546c6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="R142149ceca404b57"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="R0bd7996d44b34bcf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="Rfeb97616eef24230"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="Rba1a2f36eb154e3b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="R829eafceca0a47a1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="Re53b359504b44574"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="R589ed1d67f064ff7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="Rd8dec4f606f54fc2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="R7181e09967f9457e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="Re74b8c8d1c374897"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="R5d33b7d71b904bab"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="R89cf9888477f4c48"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="R97b1362f86464574"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="R1ff8ebdaa82c4386"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="Rf8524587a35a4995"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="Rf6ff64e335b54228"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="R8413f2d245864b9f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="R7e49e34720604698"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="R509d0b6145b64750"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="R540f57d9873b4296"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="R495bc5c4a7754759"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="R35ca62b371704712"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="Rb7ca1dadffd441a9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="R1e726436591949da"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="R925b8c8a695a478f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="R3a95aa98cec24283"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R74edbf506ec0469c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="Rf24eb7484be5446f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="R3b75166641ec4a4a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="R485afc9623d84620"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="R523fa293d7754b68"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="R9ff52b23f75d4e16"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="Rdd426d0a9d904f74"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="Rb32f8d9f8fcc4d74"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="Rfd2dcd1df4e14c48"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="R7ffcd4ebdb4446f5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="R29a9ea30fea6458e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="R5db2ddc55d844145"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="R96a091e7c991412e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="Ra49dbdb687ac4032"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="R754d10a4175a411c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="R641814176bdb4eb2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="R1b6dd6aa0f5e4f11"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="R804fa0e2a1734cd0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="R97525301f91746a2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="R89312b558c35436f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="Rd663f27777974ef2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="R0621fbb4cd024027"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="R6c69a842be4345f7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="R4eafd039727e44ab"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="Rd45392643d6d4e92"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="R958a7d056fa6406c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="R73b22c8b7ca248a7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="Rfb7eab62e1e1430e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R27c4fd4a24c54e23"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="R8d347a5f93374242"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="R4d98161182cf4c54"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="R8579f7e73ef34584"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="R7fe677a0bca446ca"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="Rab69e4bdafdb4d5b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="Rde657b3967dd474c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="Ra66b13053b944dca"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="Rcf3a7b857711481a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="R56b009cf27c54d70"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="Rc8217653f2fa4f7a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="Rf36f826533b24083"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="R5f0b162f9f9e4a09"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="R6473df4614a34918"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="R6431c9a1115d438f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="R7633deba82004bf4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="R75a9b81abc9a4fad"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="R1e6a980d713540c8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="Rf7f8becd0fe44a23"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="R892af6165bcc4899"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="Re58e3160135c4051"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="Reeaa450992fc4c7f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="R86471537a6a84105"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="R3b78731f55714953"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="Reb22704d10ad4199"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="Rb9b8028cf4d04186"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="Rd6a63d5a52fa428e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="R1f76975fd52745c2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="Rdcedc1fef0684301"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="R11836aeffa084df5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="Rc799234d306e4fb1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="R0e9d69b8107148c1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="Rcb0ad8c065fa4439"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="Rc02e361244594f72"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="Rf5830c3a233c4cf6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="Rd50d89aabd954fb5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="R9b3963c902d246f1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Update Rev F joint stack and provisional BOM
</commit_message>
<xml_diff>
--- a/outputs/20261002_reve_upper_pocket_bom/2026_BIZ-Lab_재료비관리_RevF_상부포켓검토.xlsx
+++ b/outputs/20261002_reve_upper_pocket_bom/2026_BIZ-Lab_재료비관리_RevF_상부포켓검토.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R1945be0e69a148e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R0cf60c70e86542a1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -195,7 +195,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="39">
+  <x:cellXfs count="58">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -309,6 +309,63 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="4" borderId="6" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="5" borderId="6" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="4" borderId="6" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="5" borderId="6" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="4" borderId="6" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="5" borderId="6" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="4" borderId="6" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="5" borderId="6" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="4" borderId="6" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="5" borderId="6" xfId="0" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2901,7 +2958,7 @@
           <x:t xml:space="preserve">견적 미확정</x:t>
         </x:is>
       </x:c>
-      <x:c r="I59" s="38" t="inlineStr">
+      <x:c r="I59" s="54" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">UP01A. 축 A 단품 1개. S45C/SM45C 가공 완료품 견적 후보; STEP/도면 승인, 업체 수락, 공급가·VAT·납기·결제 확인 전 발주 보류.</x:t>
         </x:is>
@@ -2939,7 +2996,7 @@
           <x:t xml:space="preserve">견적 미확정</x:t>
         </x:is>
       </x:c>
-      <x:c r="I60" s="38" t="inlineStr">
+      <x:c r="I60" s="54" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">UP01B. 축 B 단품 1개. S45C/SM45C 가공 완료품 견적 후보; STEP/도면 승인, 업체 수락, 공급가·VAT·납기·결제 확인 전 발주 보류.</x:t>
         </x:is>
@@ -2977,7 +3034,7 @@
           <x:t xml:space="preserve">견적 미확정</x:t>
         </x:is>
       </x:c>
-      <x:c r="I61" s="38" t="inlineStr">
+      <x:c r="I61" s="54" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">UP01C. 축 C 단품 1개. S45C/SM45C 가공 완료품 견적 후보; STEP/도면 승인, 업체 수락, 공급가·VAT·납기·결제 확인 전 발주 보류.</x:t>
         </x:is>
@@ -3104,11 +3161,11 @@
       </x:c>
       <x:c r="M64" s="1" t="n"/>
     </x:row>
-    <x:row r="65" s="13" customFormat="1" ht="30" customHeight="1">
+    <x:row r="65" s="13" customFormat="1" ht="48" customHeight="1">
       <x:c r="A65" t="n"/>
       <x:c r="B65" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">재료비 구매</x:t>
+          <x:t xml:space="preserve">구매 제외</x:t>
         </x:is>
       </x:c>
       <x:c r="C65" t="inlineStr">
@@ -3118,7 +3175,7 @@
       </x:c>
       <x:c r="D65" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">0.5 mm 심링</x:t>
+          <x:t xml:space="preserve">구형 볼쪽 0.5 mm 심링 (현 검토안 불필요)</x:t>
         </x:is>
       </x:c>
       <x:c r="E65" t="inlineStr">
@@ -3127,19 +3184,21 @@
         </x:is>
       </x:c>
       <x:c r="F65" t="n">
-        <x:v>12</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G65" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://kr.misumi-ec.com/vona2/detail/110302677870/?HissuCode=CIMR6-12-0.5</x:t>
         </x:is>
       </x:c>
-      <x:c r="H65" t="n">
-        <x:v>10909</x:v>
-      </x:c>
-      <x:c r="I65" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">F09. Rev E 12장/10,909원 후보 유지. 구형 상부 아이의 9장 사용 가정은 신규 포켓에 자동 승계하지 않음; 실측 적층·수량·납기 확인 전 발주 보류.</x:t>
+      <x:c r="H65" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">구형안 제외</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I65" s="54" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F09. 현 상부 볼쪽 적층 검토안에서 CIMR6-12-0.5 심 불필요. 기존 12장/공급가 10,909원은 구매·부분합에서 제외. 신규 WSSB10-6-1.5 적합성 확인 전 HOLD.</x:t>
         </x:is>
       </x:c>
       <x:c r="M65" s="1" t="n"/>
@@ -3308,7 +3367,7 @@
       <x:c r="A70" t="n"/>
       <x:c r="B70" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">기존 숫자 가격 후보 공급가 부분합 (신규 미견적 제외)</x:t>
+          <x:t xml:space="preserve">기존 숫자 가격 후보 공급가 부분합 (F09·신규 미견적 제외)</x:t>
         </x:is>
       </x:c>
       <x:c r="C70" t="n"/>
@@ -3318,7 +3377,7 @@
       <x:c r="G70" t="n"/>
       <x:c r="H70" t="n">
         <x:f>SUM(H4:H69)</x:f>
-        <x:v>2847305</x:v>
+        <x:v>2836396</x:v>
       </x:c>
       <x:c r="I70" t="n"/>
       <x:c r="M70" s="1" t="n"/>
@@ -3337,12 +3396,12 @@
       <x:c r="G71" t="n"/>
       <x:c r="H71" t="n">
         <x:f>ROUND(H70*10%,0)</x:f>
-        <x:v>284731</x:v>
+        <x:v>283640</x:v>
       </x:c>
       <x:c r="I71" t="n"/>
       <x:c r="M71" s="1" t="n"/>
     </x:row>
-    <x:row r="72" s="13" customFormat="1" ht="16.5" customHeight="1">
+    <x:row r="72" s="13" customFormat="1" ht="42" customHeight="1">
       <x:c r="A72" t="n"/>
       <x:c r="B72" t="inlineStr">
         <x:is>
@@ -3356,11 +3415,11 @@
       <x:c r="G72" t="n"/>
       <x:c r="H72" t="n">
         <x:f>SUM(H70:H71)</x:f>
-        <x:v>3132036</x:v>
-      </x:c>
-      <x:c r="I72" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Rev E 구형 후보 VAT포함 3,143,564원 대비 F08A/B·F12·F11 제외 11,528원 감소. UP01A/B/C 등 미견적은 아직 미반영.</x:t>
+        <x:v>3120036</x:v>
+      </x:c>
+      <x:c r="I72" s="54" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Rev E 구형 후보 VAT포함 3,143,564원 대비 F08A/B·F12·F11 제외 11,528원과 F09 제외 12,000원 감소. 신규 후보는 미견적.</x:t>
         </x:is>
       </x:c>
       <x:c r="M72" s="1" t="n"/>
@@ -3379,11 +3438,11 @@
       <x:c r="G73" t="n"/>
       <x:c r="H73" t="n">
         <x:f>$I$2-H72</x:f>
-        <x:v>867964</x:v>
-      </x:c>
-      <x:c r="I73" s="38" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">UP01A/B/C 및 신규 핀·와셔·PHS6 M6·장착 볼트/T너트 미견적. E링은 HCDGH 동봉(별도 구매 없음). 최종 예산 적합 UNKNOWN; 구매 보류.</x:t>
+        <x:v>879964</x:v>
+      </x:c>
+      <x:c r="I73" s="54" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">UP01A/B/C 및 신규 핀·머리쪽/볼쪽 와셔·PHS6 M6·장착 볼트/T너트 미견적. F09 12장 제외, E링은 HCDGH 동봉(별도 구매 없음). 최종 예산 적합 UNKNOWN; 구매 보류.</x:t>
         </x:is>
       </x:c>
       <x:c r="M73" s="1" t="n"/>
@@ -3400,18 +3459,18 @@
       <x:c r="M74" s="1" t="n"/>
     </x:row>
     <x:row r="75" s="13" customFormat="1" ht="26" customHeight="1">
-      <x:c r="B75" s="31" t="inlineStr">
+      <x:c r="B75" s="56" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">필수 미선정 항목</x:t>
         </x:is>
       </x:c>
-      <x:c r="C75" s="31" t="n"/>
-      <x:c r="D75" s="31" t="n"/>
-      <x:c r="E75" s="31" t="n"/>
-      <x:c r="F75" s="31" t="n"/>
-      <x:c r="G75" s="31" t="n"/>
-      <x:c r="H75" s="31" t="n"/>
-      <x:c r="I75" s="31" t="inlineStr">
+      <x:c r="C75" s="56" t="n"/>
+      <x:c r="D75" s="56" t="n"/>
+      <x:c r="E75" s="56" t="n"/>
+      <x:c r="F75" s="56" t="n"/>
+      <x:c r="G75" s="56" t="n"/>
+      <x:c r="H75" s="56" t="n"/>
+      <x:c r="I75" s="56" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">유료 구매행 미반영·HOLD</x:t>
         </x:is>
@@ -3419,42 +3478,42 @@
       <x:c r="M75" s="1" t="n"/>
     </x:row>
     <x:row r="76" s="13" customFormat="1" ht="16.5" customHeight="1">
-      <x:c r="B76" s="32" t="inlineStr">
+      <x:c r="B76" s="57" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">구분</x:t>
         </x:is>
       </x:c>
-      <x:c r="C76" s="32" t="inlineStr">
+      <x:c r="C76" s="57" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">필요성</x:t>
         </x:is>
       </x:c>
-      <x:c r="D76" s="32" t="inlineStr">
+      <x:c r="D76" s="57" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">정확 SKU</x:t>
         </x:is>
       </x:c>
-      <x:c r="E76" s="32" t="inlineStr">
+      <x:c r="E76" s="57" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">수량/포장</x:t>
         </x:is>
       </x:c>
-      <x:c r="F76" s="32" t="inlineStr">
+      <x:c r="F76" s="57" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">후보처</x:t>
         </x:is>
       </x:c>
-      <x:c r="G76" s="32" t="inlineStr">
+      <x:c r="G76" s="57" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">링크</x:t>
         </x:is>
       </x:c>
-      <x:c r="H76" s="32" t="inlineStr">
+      <x:c r="H76" s="57" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">가격</x:t>
         </x:is>
       </x:c>
-      <x:c r="I76" s="32" t="inlineStr">
+      <x:c r="I76" s="57" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">상태</x:t>
         </x:is>
@@ -3462,42 +3521,42 @@
       <x:c r="M76" s="1" t="n"/>
     </x:row>
     <x:row r="77" s="13" customFormat="1" ht="52" customHeight="1">
-      <x:c r="B77" s="33" t="inlineStr">
+      <x:c r="B77" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">신규 상부 피벗 핀</x:t>
         </x:is>
       </x:c>
-      <x:c r="C77" s="33" t="inlineStr">
+      <x:c r="C77" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">3축 포켓-아이 연결</x:t>
         </x:is>
       </x:c>
-      <x:c r="D77" s="33" t="inlineStr">
+      <x:c r="D77" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">미선정 (후보 HCDGH6-35)</x:t>
         </x:is>
       </x:c>
-      <x:c r="E77" s="33" t="inlineStr">
+      <x:c r="E77" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">3개(축당 1개), E링 각 1개 동봉</x:t>
         </x:is>
       </x:c>
-      <x:c r="F77" s="33" t="inlineStr">
+      <x:c r="F77" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">한국미스미</x:t>
         </x:is>
       </x:c>
-      <x:c r="G77" s="33" t="inlineStr">
+      <x:c r="G77" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://kr.misumi-ec.com/vona2/detail/110300095750/?HissuCode=HCDGH6-35</x:t>
         </x:is>
       </x:c>
-      <x:c r="H77" s="33" t="inlineStr">
+      <x:c r="H77" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">견적 미확정</x:t>
         </x:is>
       </x:c>
-      <x:c r="I77" s="33" t="inlineStr">
+      <x:c r="I77" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">핀 보증 항복·홈 강도·eye 공차·링 축하중 미검증 HOLD</x:t>
         </x:is>
@@ -3505,42 +3564,42 @@
       <x:c r="M77" s="1" t="n"/>
     </x:row>
     <x:row r="78" s="13" customFormat="1" ht="52" customHeight="1">
-      <x:c r="B78" s="33" t="inlineStr">
+      <x:c r="B78" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">핀 리테이너</x:t>
         </x:is>
       </x:c>
-      <x:c r="C78" s="33" t="inlineStr">
+      <x:c r="C78" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">피벗 축방향 이탈 방지</x:t>
         </x:is>
       </x:c>
-      <x:c r="D78" s="33" t="inlineStr">
+      <x:c r="D78" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">HCDGH6-35 동봉 E형 No.5 고정링</x:t>
         </x:is>
       </x:c>
-      <x:c r="E78" s="33" t="inlineStr">
+      <x:c r="E78" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">동봉 3개; 별도 발주 없음</x:t>
         </x:is>
       </x:c>
-      <x:c r="F78" s="33" t="inlineStr">
+      <x:c r="F78" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">한국미스미</x:t>
         </x:is>
       </x:c>
-      <x:c r="G78" s="33" t="inlineStr">
+      <x:c r="G78" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://kr.misumi-ec.com/vona2/detail/110300095750/?HissuCode=HCDGH6-35</x:t>
         </x:is>
       </x:c>
-      <x:c r="H78" s="33" t="inlineStr">
+      <x:c r="H78" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">동봉 (별도 발주 없음)</x:t>
         </x:is>
       </x:c>
-      <x:c r="I78" s="33" t="inlineStr">
+      <x:c r="I78" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">HCDGH에 동봉; 별도 구매 0. 실제 링 유지력 미검증 HOLD</x:t>
         </x:is>
@@ -3548,135 +3607,175 @@
       <x:c r="M78" s="1" t="n"/>
     </x:row>
     <x:row r="79" s="13" customFormat="1" ht="52" customHeight="1">
-      <x:c r="B79" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">조립 스페이서/와셔</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C79" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">축별 유격·간섭 제어</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D79" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">미선정 (후보 WSSB10-6-4; F09 CIMR6-12-0.5)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E79" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">와셔 3개; 심 명목 9장(기존 F09 12장 후보)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F79" s="33" t="inlineStr">
+      <x:c r="B79" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">머리쪽 와셔</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C79" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">핀 머리와 eye 사이의 축방향 적층</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D79" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미선정 (후보 WSSB10-6-4)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E79" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">3개(축당 1개)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F79" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">한국미스미</x:t>
         </x:is>
       </x:c>
-      <x:c r="G79" s="33" t="inlineStr">
+      <x:c r="G79" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://kr.misumi-ec.com/vona2/detail/110302677010/?HissuCode=WSSB10-6-4</x:t>
         </x:is>
       </x:c>
-      <x:c r="H79" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">신규 와셔 견적 미확정; F09 기포함</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I79" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">eye 폭·링 장착 여유 미확정. F09 심 12장과 중복 구매 금지 HOLD</x:t>
+      <x:c r="H79" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">견적 미확정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I79" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">머리쪽 T4 와셔. eye 폭·핀 릴리프·링 여유·강도 미검증 HOLD</x:t>
         </x:is>
       </x:c>
       <x:c r="M79" s="1" t="n"/>
     </x:row>
     <x:row r="80" s="13" customFormat="1" ht="52" customHeight="1">
-      <x:c r="B80" s="33" t="inlineStr">
+      <x:c r="B80" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">볼쪽 와셔</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C80" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">eye와 PHS6 볼 사이의 축방향 적층</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D80" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미선정 (후보 WSSB10-6-1.5)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E80" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">3개(축당 1개)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F80" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">한국미스미</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G80" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://kr.misumi-ec.com/vona2/detail/110302677010/?HissuCode=WSSB10-6-1.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H80" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">표시 공급가 1,470원/개 (실결제 미확정)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I80" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">OD10 ID6 T1.5±0.1. 2026-10-02 한국미스미 화면 VAT 1,617원/개·재고100·기준출하10/07 표시. 실제 결제·납기·CAD 적합 HOLD</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M80" s="1" t="n"/>
+    </x:row>
+    <x:row r="81" s="13" customFormat="1" ht="86" customHeight="1">
+      <x:c r="B81" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">PHS6 하우징 M6 포획·이탈방지</x:t>
         </x:is>
       </x:c>
-      <x:c r="C80" s="33" t="inlineStr">
+      <x:c r="C81" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">하우징 M6 유효물림·잠금 방식</x:t>
         </x:is>
       </x:c>
-      <x:c r="D80" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">미선정 (후보 PACK-SCB6-12-YBM)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E80" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">3축 3개 필요; 후보 10개입 1팩</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F80" s="33" t="inlineStr">
+      <x:c r="D81" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미선정 (후보 CBS6-12 저두볼트)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E81" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">3축 3개 필요; 최소 1개 단위</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F81" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">한국미스미</x:t>
         </x:is>
       </x:c>
-      <x:c r="G80" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://kr.misumi-ec.com/vona2/detail/110300239250/?HissuCode=PACK-SCB6-12-YBM</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H80" s="33" t="inlineStr">
+      <x:c r="G81" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://kr.misumi-ec.com/vona2/detail/110100142110/?HissuCode=CBS6-12</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H81" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">표시 공급가 671원/개 (실결제 미확정)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I81" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SCM435 10.9, M6×12·머리 Ø10×높이4. 명목 Ø11×깊이6 리세스에 머리 상면 2mm 후퇴, 3mm 웹 뒤 PHS6 공칭 물림9mm이나 공차·바닥/니플/렌치 미확인. F21 대체 금지; F17 나사고정제는 오일·나사산·토크·경화 검증 전 후보만. 2026-10-02 한국미스미 로그인 화면 재고423·참고출하10/07 표시, 결제·납기·유효물림 HOLD</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M81" s="1" t="n"/>
+    </x:row>
+    <x:row r="82" s="13" customFormat="1" ht="52" customHeight="1">
+      <x:c r="B82" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">브래킷 장착 볼트·T너트</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C82" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">3030 프레임에 3개 브래킷 장착</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D82" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미선정 (F02/F07 재사용 미확정)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E82" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">명목 볼트 6개·너트 6개; 길이·포장 미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F82" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미확정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G82" s="55" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">—</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H82" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">견적 미확정</x:t>
         </x:is>
       </x:c>
-      <x:c r="I80" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">F21/G9EA용 볼트와 구별. M6 유효물림·잠금·머리 여유·카드결제 HOLD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M80" s="1" t="n"/>
-    </x:row>
-    <x:row r="81" s="13" customFormat="1" ht="52" customHeight="1">
-      <x:c r="B81" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">브래킷 장착 볼트·T너트</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C81" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">3030 프레임에 3개 브래킷 장착</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D81" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">미선정 (F02/F07 재사용 미확정)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E81" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">명목 볼트 6개·너트 6개; 길이·포장 미정</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F81" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">미확정</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G81" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">—</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H81" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">견적 미확정</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I81" s="33" t="inlineStr">
+      <x:c r="I82" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">F02/F07 자동 전용 금지. 납품 3030 슬롯·체결력 검증 전 HOLD</x:t>
         </x:is>
       </x:c>
-      <x:c r="M81" s="1" t="n"/>
-    </x:row>
-    <x:row r="82" s="13" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="M82" s="1" t="n"/>
     </x:row>
     <x:row r="83" s="13" customFormat="1" ht="16.5" customHeight="1">
@@ -10066,73 +10165,74 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="R925b8c8a695a478f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="R3a95aa98cec24283"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R74edbf506ec0469c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="Rf24eb7484be5446f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="R3b75166641ec4a4a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="R485afc9623d84620"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="R523fa293d7754b68"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="R9ff52b23f75d4e16"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="Rdd426d0a9d904f74"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="Rb32f8d9f8fcc4d74"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="Rfd2dcd1df4e14c48"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="R7ffcd4ebdb4446f5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="R29a9ea30fea6458e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="R5db2ddc55d844145"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="R96a091e7c991412e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="Ra49dbdb687ac4032"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="R754d10a4175a411c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="R641814176bdb4eb2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="R1b6dd6aa0f5e4f11"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="R804fa0e2a1734cd0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="R97525301f91746a2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="R89312b558c35436f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="Rd663f27777974ef2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="R0621fbb4cd024027"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="R6c69a842be4345f7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="R4eafd039727e44ab"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="Rd45392643d6d4e92"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="R958a7d056fa6406c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="R73b22c8b7ca248a7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="Rfb7eab62e1e1430e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R27c4fd4a24c54e23"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="R8d347a5f93374242"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="R4d98161182cf4c54"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="R8579f7e73ef34584"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="R7fe677a0bca446ca"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="Rab69e4bdafdb4d5b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="Rde657b3967dd474c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="Ra66b13053b944dca"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="Rcf3a7b857711481a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="R56b009cf27c54d70"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="Rc8217653f2fa4f7a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="Rf36f826533b24083"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="R5f0b162f9f9e4a09"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="R6473df4614a34918"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="R6431c9a1115d438f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="R7633deba82004bf4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="R75a9b81abc9a4fad"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="R1e6a980d713540c8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="Rf7f8becd0fe44a23"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="R892af6165bcc4899"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="Re58e3160135c4051"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="Reeaa450992fc4c7f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="R86471537a6a84105"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="R3b78731f55714953"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="Reb22704d10ad4199"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="Rb9b8028cf4d04186"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="Rd6a63d5a52fa428e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="R1f76975fd52745c2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="Rdcedc1fef0684301"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="R11836aeffa084df5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="Rc799234d306e4fb1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="R0e9d69b8107148c1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="Rcb0ad8c065fa4439"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="Rc02e361244594f72"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="Rf5830c3a233c4cf6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="Rd50d89aabd954fb5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="R9b3963c902d246f1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="R583bebdc2ead422b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="R8b092207fb4c4648"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R11528b06671f43d1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="R0e621389a8834bf4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="R5a32b06550f44a4d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="R440454ab57244a41"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="R99dd07304d4f4e3a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="R69d6ba2ae1494a1d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="R2fa00ad86af34cc2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="R9460e19b2c474eca"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="R5fe8c3ce8a0a4ebb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="Rdc67069133bf42b9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="Ra5a205d90f2a4798"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="R276879a4a7694f58"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="R66a70dd196e04ed5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="R749007f327934b6d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="Rb8b0ad2035b64137"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="Re422a59a48db4f6d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="Ra2099a85bc16401f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="R8feab95e4e234803"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="R7992e7446e86459f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="Re8f25f6f604445f4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="R8e76eab69b944fbb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="Rcca0dd6a0ba64e8a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="R585f657d09f143b4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="Ra12e360f074b4913"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="R95b0d37b37314932"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="R9e3bdc4b5c49441a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="R01935129013c46e5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="R17c2fba8bb2b423b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="Rccffff3407a44119"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="R46522f3c155f473a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="R156792f41eaa4948"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="R7f5c77b5d9cc4974"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="Rdd97855161af4051"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="Rf7178fc9bbe040e1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="R9558fb1b656d4408"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="R544fa7a814564329"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="Raa2c00115d3849bf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="R979ca16a0deb44db"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="R32ec0731dfad4332"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="R058c1048d1584bf2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="R2c959f095b094112"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="Rb774e04dc9364512"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="R770c93ef9b8e4977"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="R6a12b7d9167044fc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="R0f4470fb299648a8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="R045b72fd9afb41e9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="Rf7eeec79a4a14736"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="R214bbd8e80d84ae2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="Rb63447772bb94ceb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="Raf29dd56925e4801"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="R623e0b460078424d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="R3d7d6ab47a524d3f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="R170eb765cf1d4bad"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="R67357632afe34178"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="R1b7cbd12c5af48b3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="R133af4e5a561436b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="Ra33462abe22247f9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="Rc1480935974746b1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="Re13c8e85062f472a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="Reb05327fd74f4237"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="Rcb1705258a904ab2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="R0014357085f44851"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="Rba3c69285ae14b24"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="Rf32bbcd256c64fa7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="R80bbf0ba8ffc422e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="R94743fb3b8aa437d"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>